<commit_message>
Coleta automática em 14-09-2026 22:54
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-09-2026 22:03
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 22-09-2026 22:34
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-09-2026 22:37
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 24-09-2026 22:53
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 27-09-2026 22:44
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 30-09-2026 23:22
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 02-10-2026 23:30
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 03-10-2026 22:39
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-10-2026 00:07
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-10-2026 23:44
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 10-10-2026 23:07
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 15-10-2026 22:50
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-10-2026 21:54
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 18-10-2026 22:05
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-10-2026 23:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-10-2026 22:56
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 22-10-2026 22:59
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-10-2026 22:53
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 25-10-2026 22:19
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 26-10-2026 23:31
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 27-10-2026 23:23
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 28-10-2026 23:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 30-10-2026 23:24
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>